<commit_message>
adding in breeder facilities
</commit_message>
<xml_diff>
--- a/data/NSW_properties.xlsx
+++ b/data/NSW_properties.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thaophuongl\Documents\HASTE_CODE\OutbreakSimulator\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEAC6758-9DDE-45D2-87F8-CD5C7EA8B9B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F4882D3-02ED-4D2B-B7BC-F1ADFA706C5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-105" windowWidth="29040" windowHeight="15720" xr2:uid="{E264DCFB-2E54-41D3-AA9C-B1867134B6AE}"/>
+    <workbookView xWindow="28680" yWindow="-105" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E264DCFB-2E54-41D3-AA9C-B1867134B6AE}"/>
   </bookViews>
   <sheets>
     <sheet name="PoultryAgTrack" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1437" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1689" uniqueCount="108">
   <si>
     <t>Region Type</t>
   </si>
@@ -362,6 +362,9 @@
   </si>
   <si>
     <t>Assuming there are egg processing plants, hatcheries and poultry abbatoirs in LGAs with layers (PoultryAgTrack)</t>
+  </si>
+  <si>
+    <t>breeder</t>
   </si>
 </sst>
 </file>
@@ -4553,7 +4556,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43CCC0DD-C8CB-4A03-95AB-595E73119AFB}">
-  <dimension ref="A1:E222"/>
+  <dimension ref="A1:E253"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="34.625" customWidth="1"/>
@@ -7793,132 +7796,1075 @@
       </c>
     </row>
     <row r="191" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="D191" s="3"/>
-      <c r="E191" s="3"/>
+      <c r="A191" t="s">
+        <v>4</v>
+      </c>
+      <c r="B191" t="s">
+        <v>91</v>
+      </c>
+      <c r="C191" t="s">
+        <v>107</v>
+      </c>
+      <c r="D191" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E191" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="192" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="D192" s="3"/>
-      <c r="E192" s="3"/>
-    </row>
-    <row r="193" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D193" s="3"/>
-      <c r="E193" s="3"/>
-    </row>
-    <row r="194" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D194" s="3"/>
-      <c r="E194" s="3"/>
-    </row>
-    <row r="195" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D195" s="3"/>
-      <c r="E195" s="3"/>
-    </row>
-    <row r="196" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D196" s="3"/>
-      <c r="E196" s="3"/>
-    </row>
-    <row r="197" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D197" s="3"/>
-      <c r="E197" s="3"/>
-    </row>
-    <row r="198" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D198" s="3"/>
-      <c r="E198" s="3"/>
-    </row>
-    <row r="199" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D199" s="3"/>
-      <c r="E199" s="3"/>
-    </row>
-    <row r="200" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D200" s="3"/>
-      <c r="E200" s="3"/>
-    </row>
-    <row r="201" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D201" s="3"/>
-      <c r="E201" s="3"/>
-    </row>
-    <row r="202" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D202" s="3"/>
-      <c r="E202" s="3"/>
-    </row>
-    <row r="203" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D203" s="3"/>
-      <c r="E203" s="3"/>
-    </row>
-    <row r="204" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D204" s="3"/>
-      <c r="E204" s="3"/>
-    </row>
-    <row r="205" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D205" s="3"/>
-      <c r="E205" s="3"/>
-    </row>
-    <row r="206" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D206" s="3"/>
-      <c r="E206" s="3"/>
-    </row>
-    <row r="207" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D207" s="3"/>
-      <c r="E207" s="3"/>
-    </row>
-    <row r="208" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D208" s="3"/>
-      <c r="E208" s="3"/>
-    </row>
-    <row r="209" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D209" s="3"/>
-      <c r="E209" s="3"/>
-    </row>
-    <row r="210" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D210" s="3"/>
-      <c r="E210" s="3"/>
-    </row>
-    <row r="211" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D211" s="3"/>
-      <c r="E211" s="3"/>
-    </row>
-    <row r="212" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D212" s="3"/>
-      <c r="E212" s="3"/>
-    </row>
-    <row r="213" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D213" s="3"/>
-      <c r="E213" s="3"/>
-    </row>
-    <row r="214" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D214" s="3"/>
-      <c r="E214" s="3"/>
-    </row>
-    <row r="215" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D215" s="3"/>
-      <c r="E215" s="3"/>
-    </row>
-    <row r="216" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D216" s="3"/>
-      <c r="E216" s="3"/>
-    </row>
-    <row r="217" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D217" s="3"/>
-      <c r="E217" s="3"/>
-    </row>
-    <row r="218" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D218" s="3"/>
-      <c r="E218" s="3"/>
-    </row>
-    <row r="219" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D219" s="3"/>
-      <c r="E219" s="3"/>
-    </row>
-    <row r="220" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D220" s="3"/>
-      <c r="E220" s="3"/>
-    </row>
-    <row r="221" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D221" s="3"/>
-      <c r="E221" s="3"/>
-    </row>
-    <row r="222" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D222" s="3"/>
-      <c r="E222" s="3"/>
+      <c r="A192" t="s">
+        <v>4</v>
+      </c>
+      <c r="B192" t="s">
+        <v>6</v>
+      </c>
+      <c r="C192" t="s">
+        <v>107</v>
+      </c>
+      <c r="D192" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E192" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="193" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A193" t="s">
+        <v>4</v>
+      </c>
+      <c r="B193" t="s">
+        <v>92</v>
+      </c>
+      <c r="C193" t="s">
+        <v>107</v>
+      </c>
+      <c r="D193" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E193" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="194" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A194" t="s">
+        <v>4</v>
+      </c>
+      <c r="B194" t="s">
+        <v>9</v>
+      </c>
+      <c r="C194" t="s">
+        <v>107</v>
+      </c>
+      <c r="D194" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E194" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A195" t="s">
+        <v>4</v>
+      </c>
+      <c r="B195" t="s">
+        <v>11</v>
+      </c>
+      <c r="C195" t="s">
+        <v>107</v>
+      </c>
+      <c r="D195" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E195" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A196" t="s">
+        <v>4</v>
+      </c>
+      <c r="B196" t="s">
+        <v>14</v>
+      </c>
+      <c r="C196" t="s">
+        <v>107</v>
+      </c>
+      <c r="D196" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E196" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="197" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A197" t="s">
+        <v>4</v>
+      </c>
+      <c r="B197" t="s">
+        <v>17</v>
+      </c>
+      <c r="C197" t="s">
+        <v>107</v>
+      </c>
+      <c r="D197" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E197" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="198" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A198" t="s">
+        <v>4</v>
+      </c>
+      <c r="B198" t="s">
+        <v>18</v>
+      </c>
+      <c r="C198" t="s">
+        <v>107</v>
+      </c>
+      <c r="D198" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E198" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A199" t="s">
+        <v>4</v>
+      </c>
+      <c r="B199" t="s">
+        <v>19</v>
+      </c>
+      <c r="C199" t="s">
+        <v>107</v>
+      </c>
+      <c r="D199" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E199" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="200" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A200" t="s">
+        <v>4</v>
+      </c>
+      <c r="B200" t="s">
+        <v>20</v>
+      </c>
+      <c r="C200" t="s">
+        <v>107</v>
+      </c>
+      <c r="D200" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E200" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="201" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A201" t="s">
+        <v>4</v>
+      </c>
+      <c r="B201" t="s">
+        <v>22</v>
+      </c>
+      <c r="C201" t="s">
+        <v>107</v>
+      </c>
+      <c r="D201" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E201" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="202" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A202" t="s">
+        <v>4</v>
+      </c>
+      <c r="B202" t="s">
+        <v>23</v>
+      </c>
+      <c r="C202" t="s">
+        <v>107</v>
+      </c>
+      <c r="D202" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E202" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="203" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A203" t="s">
+        <v>4</v>
+      </c>
+      <c r="B203" t="s">
+        <v>24</v>
+      </c>
+      <c r="C203" t="s">
+        <v>107</v>
+      </c>
+      <c r="D203" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E203" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="204" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A204" t="s">
+        <v>4</v>
+      </c>
+      <c r="B204" t="s">
+        <v>25</v>
+      </c>
+      <c r="C204" t="s">
+        <v>107</v>
+      </c>
+      <c r="D204" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E204" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="205" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A205" t="s">
+        <v>4</v>
+      </c>
+      <c r="B205" t="s">
+        <v>93</v>
+      </c>
+      <c r="C205" t="s">
+        <v>107</v>
+      </c>
+      <c r="D205" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E205" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="206" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A206" t="s">
+        <v>4</v>
+      </c>
+      <c r="B206" t="s">
+        <v>27</v>
+      </c>
+      <c r="C206" t="s">
+        <v>107</v>
+      </c>
+      <c r="D206" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E206" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="207" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A207" t="s">
+        <v>4</v>
+      </c>
+      <c r="B207" t="s">
+        <v>94</v>
+      </c>
+      <c r="C207" t="s">
+        <v>107</v>
+      </c>
+      <c r="D207" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E207" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="208" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A208" t="s">
+        <v>4</v>
+      </c>
+      <c r="B208" t="s">
+        <v>29</v>
+      </c>
+      <c r="C208" t="s">
+        <v>107</v>
+      </c>
+      <c r="D208" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E208" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="209" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A209" t="s">
+        <v>4</v>
+      </c>
+      <c r="B209" t="s">
+        <v>30</v>
+      </c>
+      <c r="C209" t="s">
+        <v>107</v>
+      </c>
+      <c r="D209" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E209" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="210" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A210" t="s">
+        <v>4</v>
+      </c>
+      <c r="B210" t="s">
+        <v>33</v>
+      </c>
+      <c r="C210" t="s">
+        <v>107</v>
+      </c>
+      <c r="D210" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E210" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="211" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A211" t="s">
+        <v>4</v>
+      </c>
+      <c r="B211" t="s">
+        <v>36</v>
+      </c>
+      <c r="C211" t="s">
+        <v>107</v>
+      </c>
+      <c r="D211" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E211" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="212" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A212" t="s">
+        <v>4</v>
+      </c>
+      <c r="B212" t="s">
+        <v>37</v>
+      </c>
+      <c r="C212" t="s">
+        <v>107</v>
+      </c>
+      <c r="D212" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E212" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="213" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A213" t="s">
+        <v>4</v>
+      </c>
+      <c r="B213" t="s">
+        <v>96</v>
+      </c>
+      <c r="C213" t="s">
+        <v>107</v>
+      </c>
+      <c r="D213" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E213" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="214" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A214" t="s">
+        <v>4</v>
+      </c>
+      <c r="B214" t="s">
+        <v>40</v>
+      </c>
+      <c r="C214" t="s">
+        <v>107</v>
+      </c>
+      <c r="D214" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E214" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="215" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A215" t="s">
+        <v>4</v>
+      </c>
+      <c r="B215" t="s">
+        <v>41</v>
+      </c>
+      <c r="C215" t="s">
+        <v>107</v>
+      </c>
+      <c r="D215" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E215" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="216" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A216" t="s">
+        <v>4</v>
+      </c>
+      <c r="B216" t="s">
+        <v>43</v>
+      </c>
+      <c r="C216" t="s">
+        <v>107</v>
+      </c>
+      <c r="D216" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E216" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="217" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A217" t="s">
+        <v>4</v>
+      </c>
+      <c r="B217" t="s">
+        <v>47</v>
+      </c>
+      <c r="C217" t="s">
+        <v>107</v>
+      </c>
+      <c r="D217" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E217" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="218" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A218" t="s">
+        <v>4</v>
+      </c>
+      <c r="B218" t="s">
+        <v>48</v>
+      </c>
+      <c r="C218" t="s">
+        <v>107</v>
+      </c>
+      <c r="D218" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E218" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="219" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A219" t="s">
+        <v>4</v>
+      </c>
+      <c r="B219" t="s">
+        <v>49</v>
+      </c>
+      <c r="C219" t="s">
+        <v>107</v>
+      </c>
+      <c r="D219" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E219" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="220" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A220" t="s">
+        <v>4</v>
+      </c>
+      <c r="B220" t="s">
+        <v>50</v>
+      </c>
+      <c r="C220" t="s">
+        <v>107</v>
+      </c>
+      <c r="D220" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E220" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="221" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A221" t="s">
+        <v>4</v>
+      </c>
+      <c r="B221" t="s">
+        <v>51</v>
+      </c>
+      <c r="C221" t="s">
+        <v>107</v>
+      </c>
+      <c r="D221" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E221" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="222" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A222" t="s">
+        <v>4</v>
+      </c>
+      <c r="B222" t="s">
+        <v>52</v>
+      </c>
+      <c r="C222" t="s">
+        <v>107</v>
+      </c>
+      <c r="D222" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E222" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="223" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A223" t="s">
+        <v>4</v>
+      </c>
+      <c r="B223" t="s">
+        <v>53</v>
+      </c>
+      <c r="C223" t="s">
+        <v>107</v>
+      </c>
+      <c r="D223" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E223" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="224" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A224" t="s">
+        <v>4</v>
+      </c>
+      <c r="B224" t="s">
+        <v>54</v>
+      </c>
+      <c r="C224" t="s">
+        <v>107</v>
+      </c>
+      <c r="D224" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E224" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="225" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A225" t="s">
+        <v>4</v>
+      </c>
+      <c r="B225" t="s">
+        <v>56</v>
+      </c>
+      <c r="C225" t="s">
+        <v>107</v>
+      </c>
+      <c r="D225" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E225" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="226" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A226" t="s">
+        <v>4</v>
+      </c>
+      <c r="B226" t="s">
+        <v>57</v>
+      </c>
+      <c r="C226" t="s">
+        <v>107</v>
+      </c>
+      <c r="D226" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E226" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="227" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A227" t="s">
+        <v>4</v>
+      </c>
+      <c r="B227" t="s">
+        <v>98</v>
+      </c>
+      <c r="C227" t="s">
+        <v>107</v>
+      </c>
+      <c r="D227" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E227" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="228" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A228" t="s">
+        <v>4</v>
+      </c>
+      <c r="B228" t="s">
+        <v>58</v>
+      </c>
+      <c r="C228" t="s">
+        <v>107</v>
+      </c>
+      <c r="D228" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E228" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="229" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A229" t="s">
+        <v>4</v>
+      </c>
+      <c r="B229" t="s">
+        <v>61</v>
+      </c>
+      <c r="C229" t="s">
+        <v>107</v>
+      </c>
+      <c r="D229" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E229" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="230" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A230" t="s">
+        <v>4</v>
+      </c>
+      <c r="B230" t="s">
+        <v>62</v>
+      </c>
+      <c r="C230" t="s">
+        <v>107</v>
+      </c>
+      <c r="D230" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E230" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="231" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A231" t="s">
+        <v>4</v>
+      </c>
+      <c r="B231" t="s">
+        <v>63</v>
+      </c>
+      <c r="C231" t="s">
+        <v>107</v>
+      </c>
+      <c r="D231" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E231" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="232" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A232" t="s">
+        <v>4</v>
+      </c>
+      <c r="B232" t="s">
+        <v>64</v>
+      </c>
+      <c r="C232" t="s">
+        <v>107</v>
+      </c>
+      <c r="D232" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E232" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="233" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A233" t="s">
+        <v>4</v>
+      </c>
+      <c r="B233" t="s">
+        <v>65</v>
+      </c>
+      <c r="C233" t="s">
+        <v>107</v>
+      </c>
+      <c r="D233" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E233" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="234" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A234" t="s">
+        <v>4</v>
+      </c>
+      <c r="B234" t="s">
+        <v>66</v>
+      </c>
+      <c r="C234" t="s">
+        <v>107</v>
+      </c>
+      <c r="D234" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E234" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="235" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A235" t="s">
+        <v>4</v>
+      </c>
+      <c r="B235" t="s">
+        <v>67</v>
+      </c>
+      <c r="C235" t="s">
+        <v>107</v>
+      </c>
+      <c r="D235" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E235" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="236" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A236" t="s">
+        <v>4</v>
+      </c>
+      <c r="B236" t="s">
+        <v>99</v>
+      </c>
+      <c r="C236" t="s">
+        <v>107</v>
+      </c>
+      <c r="D236" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E236" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="237" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A237" t="s">
+        <v>4</v>
+      </c>
+      <c r="B237" t="s">
+        <v>68</v>
+      </c>
+      <c r="C237" t="s">
+        <v>107</v>
+      </c>
+      <c r="D237" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E237" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="238" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A238" t="s">
+        <v>4</v>
+      </c>
+      <c r="B238" t="s">
+        <v>69</v>
+      </c>
+      <c r="C238" t="s">
+        <v>107</v>
+      </c>
+      <c r="D238" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E238" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="239" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A239" t="s">
+        <v>4</v>
+      </c>
+      <c r="B239" t="s">
+        <v>70</v>
+      </c>
+      <c r="C239" t="s">
+        <v>107</v>
+      </c>
+      <c r="D239" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E239" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="240" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A240" t="s">
+        <v>4</v>
+      </c>
+      <c r="B240" t="s">
+        <v>100</v>
+      </c>
+      <c r="C240" t="s">
+        <v>107</v>
+      </c>
+      <c r="D240" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E240" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="241" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A241" t="s">
+        <v>4</v>
+      </c>
+      <c r="B241" t="s">
+        <v>101</v>
+      </c>
+      <c r="C241" t="s">
+        <v>107</v>
+      </c>
+      <c r="D241" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E241" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="242" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A242" t="s">
+        <v>4</v>
+      </c>
+      <c r="B242" t="s">
+        <v>72</v>
+      </c>
+      <c r="C242" t="s">
+        <v>107</v>
+      </c>
+      <c r="D242" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E242" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="243" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A243" t="s">
+        <v>4</v>
+      </c>
+      <c r="B243" t="s">
+        <v>73</v>
+      </c>
+      <c r="C243" t="s">
+        <v>107</v>
+      </c>
+      <c r="D243" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E243" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="244" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A244" t="s">
+        <v>4</v>
+      </c>
+      <c r="B244" t="s">
+        <v>102</v>
+      </c>
+      <c r="C244" t="s">
+        <v>107</v>
+      </c>
+      <c r="D244" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E244" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="245" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A245" t="s">
+        <v>4</v>
+      </c>
+      <c r="B245" t="s">
+        <v>74</v>
+      </c>
+      <c r="C245" t="s">
+        <v>107</v>
+      </c>
+      <c r="D245" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E245" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="246" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A246" t="s">
+        <v>4</v>
+      </c>
+      <c r="B246" t="s">
+        <v>103</v>
+      </c>
+      <c r="C246" t="s">
+        <v>107</v>
+      </c>
+      <c r="D246" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E246" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="247" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A247" t="s">
+        <v>4</v>
+      </c>
+      <c r="B247" t="s">
+        <v>104</v>
+      </c>
+      <c r="C247" t="s">
+        <v>107</v>
+      </c>
+      <c r="D247" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E247" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="248" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A248" t="s">
+        <v>4</v>
+      </c>
+      <c r="B248" t="s">
+        <v>75</v>
+      </c>
+      <c r="C248" t="s">
+        <v>107</v>
+      </c>
+      <c r="D248" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E248" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="249" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A249" t="s">
+        <v>4</v>
+      </c>
+      <c r="B249" t="s">
+        <v>76</v>
+      </c>
+      <c r="C249" t="s">
+        <v>107</v>
+      </c>
+      <c r="D249" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E249" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="250" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A250" t="s">
+        <v>4</v>
+      </c>
+      <c r="B250" t="s">
+        <v>77</v>
+      </c>
+      <c r="C250" t="s">
+        <v>107</v>
+      </c>
+      <c r="D250" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E250" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="251" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A251" t="s">
+        <v>4</v>
+      </c>
+      <c r="B251" t="s">
+        <v>78</v>
+      </c>
+      <c r="C251" t="s">
+        <v>107</v>
+      </c>
+      <c r="D251" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E251" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="252" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A252" t="s">
+        <v>4</v>
+      </c>
+      <c r="B252" t="s">
+        <v>79</v>
+      </c>
+      <c r="C252" t="s">
+        <v>107</v>
+      </c>
+      <c r="D252" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E252" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="253" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A253" t="s">
+        <v>4</v>
+      </c>
+      <c r="B253" t="s">
+        <v>80</v>
+      </c>
+      <c r="C253" t="s">
+        <v>107</v>
+      </c>
+      <c r="D253" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E253" s="3">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>